<commit_message>
Added chessboard_calibration_node.py Added/modified image_data_simulator_node.py Started moving to Claude Code Pro (NTD6900/year)
</commit_message>
<xml_diff>
--- a/samples/calibration01/stereo_calib.xlsx
+++ b/samples/calibration01/stereo_calib.xlsx
@@ -816,7 +816,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>image_1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>image_1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>image_1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>